<commit_message>
Corrección de bug en el anonimizador y actualizando datasets anonimizados
</commit_message>
<xml_diff>
--- a/datasets/2025_2T/estadisticas_FP_P01.xlsx
+++ b/datasets/2025_2T/estadisticas_FP_P01.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,227 +434,243 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>SIT_1, 2 o 3</t>
+          <t>SIT</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>PARCIAL_100</t>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>EXAMEN 1E_100</t>
+          <t>EXAMEN 1E</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>TEMA 1E-1_25</t>
+          <t>TEMA 1E-1</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>TEMA 1E-2_25</t>
+          <t>TEMA 1E-2</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>TEMA 1E-3_25</t>
+          <t>TEMA 1E-3</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>TEMA 1E-4_25</t>
+          <t>TEMA 1E-4</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>ESTADO 1E_1, 2 o 3</t>
+          <t>ESTADO 1E</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>REVISADO_X_ESTUDIANTE 1E_0 o 1</t>
+          <t>REVISADO_X_ESTUDIANTE 1E</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>FINAL_100</t>
+          <t>FINAL</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>EXAMEN 2E_100</t>
+          <t>EXAMEN 2E</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>TEMA 2E-1_30</t>
+          <t>TEMA 2E-1</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>TEMA 2E-2_35</t>
+          <t>TEMA 2E-2</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>TEMA 2E-3_35</t>
+          <t>TEMA 2E-3</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>ESTADO 2E_1, 2 o 3</t>
+          <t>ESTADO 2E</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>REVISADO_X_ESTUDIANTE 2E_0 o 1</t>
+          <t>REVISADO_X_ESTUDIANTE 2E</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>MEJORAMIENTO_100</t>
+          <t>MEJORAMIENTO</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>EXAMEN 3E_100</t>
+          <t>EXAMEN 3E</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>TEMA 3E-1_20</t>
+          <t>TEMA 3E-1</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>TEMA 3E-2_30</t>
+          <t>TEMA 3E-2</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>TEMA 3E-3_50</t>
+          <t>TEMA 3E-3</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>ESTADO 3E_1, 2 o 3</t>
+          <t>ESTADO 3E</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>REVISADO_X_ESTUDIANTE 3E_0 o 1</t>
+          <t>REVISADO_X_ESTUDIANTE 3E</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>PRACTICO_100</t>
+          <t>PRACTICO</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>TALLERES_80</t>
+          <t>TALLERES</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>PARTICIPACION_20</t>
+          <t>PARTICIPACION</t>
         </is>
       </c>
       <c r="AD1" t="inlineStr">
         <is>
-          <t>TRABAJOS_EXTRA_0 o 1</t>
+          <t>TRABAJOS_EXTRA</t>
         </is>
       </c>
       <c r="AE1" t="inlineStr">
         <is>
-          <t>ESTADO_AP, RP o PF</t>
+          <t>ESTADO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>199835244</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Unnamed: 0_level_1</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Camila Paredes</t>
+          <t>Unnamed: 1_level_1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CI-029</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
+          <t>Unnamed: 2_level_1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1, 2 o 3</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>56</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>49</v>
+        <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="H2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I2" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="J2" t="n">
-        <v>15</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1</v>
+        <v>25</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>1, 2 o 3</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0 o 1</t>
+        </is>
       </c>
       <c r="M2" t="n">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="N2" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="O2" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="P2" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="Q2" t="n">
+        <v>35</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>1, 2 o 3</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>0 o 1</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>100</v>
+      </c>
+      <c r="U2" t="n">
+        <v>100</v>
+      </c>
+      <c r="V2" t="n">
+        <v>20</v>
+      </c>
+      <c r="W2" t="n">
         <v>30</v>
       </c>
-      <c r="R2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0</v>
-      </c>
       <c r="X2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
+        <v>50</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>1, 2 o 3</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>0 o 1</t>
+        </is>
       </c>
       <c r="AA2" t="n">
         <v>100</v>
@@ -665,49 +681,51 @@
       <c r="AC2" t="n">
         <v>20</v>
       </c>
-      <c r="AD2" t="n">
-        <v>0</v>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>0 o 1</t>
+        </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>AP, RP o PF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>199558370</v>
+        <v>199835244</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Miguel Miranda</t>
+          <t>Camila Paredes</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LI-004</t>
+          <t>CI-029</t>
         </is>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="F3" t="n">
+        <v>49</v>
+      </c>
+      <c r="G3" t="n">
         <v>4</v>
       </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="K3" t="n">
         <v>1</v>
@@ -716,25 +734,25 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="R3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
@@ -758,159 +776,159 @@
         <v>0</v>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB3" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="AC3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="AD3" t="n">
         <v>0</v>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>PF</t>
+          <t>AP</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>199513113</v>
+        <v>199558370</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nuria Escobar</t>
+          <t>Miguel Miranda</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LI-008</t>
+          <t>LI-004</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
         <v>2</v>
       </c>
-      <c r="H4" t="n">
-        <v>3</v>
-      </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
         <v>2</v>
       </c>
-      <c r="J4" t="n">
-        <v>7</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" t="n">
-        <v>63</v>
-      </c>
-      <c r="N4" t="n">
-        <v>36</v>
-      </c>
-      <c r="O4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P4" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>29</v>
-      </c>
-      <c r="R4" t="n">
-        <v>1</v>
-      </c>
       <c r="S4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z4" t="n">
         <v>0</v>
       </c>
       <c r="AA4" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="AB4" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="AC4" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="AD4" t="n">
         <v>0</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>PF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>199888787</v>
+        <v>199513113</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Guillermo Flores</t>
+          <t>Nuria Escobar</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CI-029</t>
+          <t>LI-008</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="F5" t="n">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="G5" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="n">
         <v>7</v>
       </c>
-      <c r="J5" t="n">
-        <v>23</v>
-      </c>
       <c r="K5" t="n">
         <v>1</v>
       </c>
@@ -918,19 +936,19 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="N5" t="n">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="O5" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="P5" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="Q5" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="R5" t="n">
         <v>1</v>
@@ -939,34 +957,34 @@
         <v>1</v>
       </c>
       <c r="T5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="W5" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X5" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="Y5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z5" t="n">
         <v>0</v>
       </c>
       <c r="AA5" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="AB5" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="AC5" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="AD5" t="n">
         <v>0</v>
@@ -979,11 +997,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>199644195</v>
+        <v>199888787</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nicolás Carrillo</t>
+          <t>Guillermo Flores</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -995,43 +1013,43 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="F6" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="G6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J6" t="n">
+        <v>23</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>80</v>
+      </c>
+      <c r="N6" t="n">
+        <v>70</v>
+      </c>
+      <c r="O6" t="n">
         <v>25</v>
       </c>
-      <c r="H6" t="n">
-        <v>23</v>
-      </c>
-      <c r="I6" t="n">
-        <v>9</v>
-      </c>
-      <c r="J6" t="n">
-        <v>19</v>
-      </c>
-      <c r="K6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" t="n">
-        <v>100</v>
-      </c>
-      <c r="N6" t="n">
-        <v>100</v>
-      </c>
-      <c r="O6" t="n">
-        <v>30</v>
-      </c>
       <c r="P6" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="Q6" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="R6" t="n">
         <v>1</v>
@@ -1080,38 +1098,38 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>199628394</v>
+        <v>199644195</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Guillermo Johnson</t>
+          <t>Nicolás Carrillo</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CI-013</t>
+          <t>CI-029</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="F7" t="n">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="G7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H7" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I7" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="J7" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K7" t="n">
         <v>1</v>
@@ -1120,19 +1138,19 @@
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="N7" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="O7" t="n">
         <v>30</v>
       </c>
       <c r="P7" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="Q7" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R7" t="n">
         <v>1</v>
@@ -1162,10 +1180,10 @@
         <v>0</v>
       </c>
       <c r="AA7" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AB7" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="AC7" t="n">
         <v>20</v>
@@ -1181,65 +1199,65 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>199617027</v>
+        <v>199628394</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nicolás Benítez</t>
+          <t>Guillermo Johnson</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LI-001</t>
+          <t>CI-013</t>
         </is>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>20</v>
+        <v>86</v>
       </c>
       <c r="F8" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="H8" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="I8" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="R8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T8" t="n">
         <v>0</v>
@@ -1263,158 +1281,158 @@
         <v>0</v>
       </c>
       <c r="AA8" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="AB8" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="AC8" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="AD8" t="n">
         <v>0</v>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>PF</t>
+          <t>AP</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>199573159</v>
+        <v>199617027</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Inés Pérez</t>
+          <t>Nicolás Benítez</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CI-015</t>
+          <t>LI-001</t>
         </is>
       </c>
       <c r="D9" t="n">
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>94</v>
+        <v>20</v>
       </c>
       <c r="F9" t="n">
-        <v>92</v>
+        <v>14</v>
       </c>
       <c r="G9" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="H9" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I9" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="J9" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="W9" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Y9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z9" t="n">
         <v>0</v>
       </c>
       <c r="AA9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AB9" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="AC9" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="AD9" t="n">
         <v>0</v>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>PF</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>199886124</v>
+        <v>199573159</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Óscar Rivas</t>
+          <t>Inés Pérez</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LI-008</t>
+          <t>CI-015</t>
         </is>
       </c>
       <c r="D10" t="n">
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="F10" t="n">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="H10" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="I10" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="J10" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="K10" t="n">
         <v>1</v>
@@ -1423,19 +1441,19 @@
         <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="N10" t="n">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="O10" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="P10" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="Q10" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R10" t="n">
         <v>1</v>
@@ -1444,19 +1462,19 @@
         <v>1</v>
       </c>
       <c r="T10" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="U10" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="V10" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="W10" t="n">
         <v>30</v>
       </c>
       <c r="X10" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="Y10" t="n">
         <v>1</v>
@@ -1484,100 +1502,201 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>199553737</v>
+        <v>199886124</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Raúl Mendoza</t>
+          <t>Óscar Rivas</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CI-013</t>
+          <t>LI-008</t>
         </is>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F11" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G11" t="n">
         <v>3</v>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I11" t="n">
         <v>10</v>
       </c>
       <c r="J11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>76</v>
+      </c>
+      <c r="N11" t="n">
+        <v>62</v>
+      </c>
+      <c r="O11" t="n">
+        <v>16</v>
+      </c>
+      <c r="P11" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>31</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" t="n">
+        <v>94</v>
+      </c>
+      <c r="U11" t="n">
+        <v>94</v>
+      </c>
+      <c r="V11" t="n">
+        <v>18</v>
+      </c>
+      <c r="W11" t="n">
+        <v>30</v>
+      </c>
+      <c r="X11" t="n">
+        <v>46</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>80</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>20</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>199553737</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Raúl Mendoza</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CI-013</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>35</v>
+      </c>
+      <c r="F12" t="n">
+        <v>24</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" t="n">
+        <v>10</v>
+      </c>
+      <c r="J12" t="n">
         <v>9</v>
       </c>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
-      <c r="M11" t="n">
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
         <v>55</v>
       </c>
-      <c r="N11" t="n">
+      <c r="N12" t="n">
         <v>50</v>
       </c>
-      <c r="O11" t="n">
-        <v>1</v>
-      </c>
-      <c r="P11" t="n">
+      <c r="O12" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" t="n">
         <v>16</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="Q12" t="n">
         <v>33</v>
       </c>
-      <c r="R11" t="n">
-        <v>1</v>
-      </c>
-      <c r="S11" t="n">
-        <v>1</v>
-      </c>
-      <c r="T11" t="n">
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="n">
+        <v>1</v>
+      </c>
+      <c r="T12" t="n">
         <v>50</v>
       </c>
-      <c r="U11" t="n">
+      <c r="U12" t="n">
         <v>50</v>
       </c>
-      <c r="V11" t="n">
+      <c r="V12" t="n">
         <v>13</v>
       </c>
-      <c r="W11" t="n">
+      <c r="W12" t="n">
         <v>13</v>
       </c>
-      <c r="X11" t="n">
+      <c r="X12" t="n">
         <v>24</v>
       </c>
-      <c r="Y11" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA11" t="n">
+      <c r="Y12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="n">
         <v>90</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AB12" t="n">
         <v>72</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AC12" t="n">
         <v>18</v>
       </c>
-      <c r="AD11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE11" t="inlineStr">
+      <c r="AD12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" t="inlineStr">
         <is>
           <t>AP</t>
         </is>

</xml_diff>